<commit_message>
new bootloader TWI commands and handling, new TWI status struct, some code cleanup and optimizations
</commit_message>
<xml_diff>
--- a/docs/ESP32 Pins.xlsx
+++ b/docs/ESP32 Pins.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="32160" windowHeight="15165"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="32160" windowHeight="15165"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="467" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="194">
   <si>
     <t>OK</t>
   </si>
@@ -1111,7 +1111,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="114">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1451,6 +1451,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1461,6 +1464,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFFFF99"/>
       <color rgb="FFFF7D7D"/>
       <color rgb="FFF7AFDD"/>
       <color rgb="FFFBD5ED"/>
@@ -1917,7 +1921,7 @@
       <c r="C5" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="114" t="s">
         <v>191</v>
       </c>
       <c r="E5" s="5"/>
@@ -2520,7 +2524,7 @@
       <c r="C18" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D18" s="8" t="s">
+      <c r="D18" s="114" t="s">
         <v>185</v>
       </c>
       <c r="E18" s="113"/>
@@ -2609,9 +2613,7 @@
         <v>0</v>
       </c>
       <c r="D20" s="8"/>
-      <c r="E20" s="17" t="s">
-        <v>50</v>
-      </c>
+      <c r="E20" s="17"/>
       <c r="F20" s="8" t="s">
         <v>56</v>
       </c>
@@ -2640,7 +2642,7 @@
       <c r="C21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D21" s="8" t="s">
+      <c r="D21" s="114" t="s">
         <v>189</v>
       </c>
       <c r="E21" s="17"/>
@@ -2670,7 +2672,7 @@
       <c r="C22" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D22" s="8" t="s">
+      <c r="D22" s="114" t="s">
         <v>193</v>
       </c>
       <c r="E22" s="17"/>
@@ -2747,7 +2749,7 @@
       <c r="C25" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D25" s="8" t="s">
+      <c r="D25" s="114" t="s">
         <v>184</v>
       </c>
       <c r="E25" s="17"/>
@@ -2873,7 +2875,7 @@
       <c r="C29" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="114" t="s">
         <v>187</v>
       </c>
       <c r="E29" s="17"/>

</xml_diff>